<commit_message>
Fix duplicate citation candidates from merged references and Excel template tables
</commit_message>
<xml_diff>
--- a/templates/UNEP/引用采集模板.xlsx
+++ b/templates/UNEP/引用采集模板.xlsx
@@ -102,7 +102,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="T1" displayName="T1" ref="A1:AC101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CitationRecords" displayName="CitationRecords" ref="A1:AC101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="29">
     <x:tableColumn id="1" name="记录编号*"/>
     <x:tableColumn id="2" name="论文编号*"/>
@@ -139,7 +139,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="T2" displayName="T2" ref="A1:P101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PaperInfo" displayName="PaperInfo" ref="A1:P101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="论文编号*"/>
     <x:tableColumn id="2" name="题名原文*"/>
@@ -163,7 +163,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="T3" displayName="T3" ref="A1:K101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReportInfo" displayName="ReportInfo" ref="A1:K101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="报告编号*"/>
     <x:tableColumn id="2" name="发布组织*"/>
@@ -182,7 +182,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="T4" displayName="T4" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="EntryExamples" displayName="EntryExamples" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="记录编号"/>
     <x:tableColumn id="2" name="论文编号"/>
@@ -201,7 +201,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="T5" displayName="T5" ref="A1:B21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Instructions" displayName="Instructions" ref="A1:B21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="项目"/>
     <x:tableColumn id="2" name="填写规则"/>

</xml_diff>